<commit_message>
Fix: added pydantic settings config and env support
</commit_message>
<xml_diff>
--- a/data/accounts_registry.xlsx
+++ b/data/accounts_registry.xlsx
@@ -489,42 +489,42 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>rjrrk ej'</t>
+          <t>3tt3t3t3t</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+77700042874</t>
+          <t>+77004287470</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Работник</t>
+          <t>Выпускник</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Инженерные технологии</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>6B11380 - Вычислительная техника и программное обеспечение</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>vtpo 25-</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>pending</t>
         </is>
       </c>
     </row>

</xml_diff>